<commit_message>
Add the 실습 4 Excel workbook and live KPI rows.
The workbook follows the lecture: masters, practice formulas, a monthly dashboard, and a short report.
</commit_message>
<xml_diff>
--- a/오늘마감_KPI.xlsx
+++ b/오늘마감_KPI.xlsx
@@ -120,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -159,6 +159,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -253,7 +254,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -1313,7 +1313,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1339,15 +1339,227 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>visit</t>
         </is>
       </c>
-      <c r="B2" s="17" t="inlineStr"/>
-      <c r="C2" s="16" t="inlineStr">
-        <is>
-          <t>사이트의 KPI 내려받기 CSV를 여기부터 붙여넣는다</t>
+      <c r="B2" s="18" t="inlineStr"/>
+      <c r="C2" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-16T22:57:18.055+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="18" t="inlineStr">
+        <is>
+          <t>complete_item</t>
+        </is>
+      </c>
+      <c r="B3" s="18" t="inlineStr">
+        <is>
+          <t>과제</t>
+        </is>
+      </c>
+      <c r="C3" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-16T22:57:48.488+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>visit</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr"/>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-16T22:57:49.844+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>visit</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr"/>
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-16T22:59:12.013483+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>visit</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr"/>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-16T22:59:12.442+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>today_cleared</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr"/>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-16T22:59:13.71+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>visit</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr"/>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-16T22:59:15.168+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>visit</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr"/>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-16T23:02:08.002+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>visit</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr"/>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-16T23:02:09.403+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>visit</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr"/>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-16T23:02:52.569+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>visit</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr"/>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-16T23:03:13.741+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>visit</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr"/>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-16T23:12:08.226+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>visit</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr"/>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-16T23:12:08.608+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>visit</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr"/>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-16T23:12:50.07+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>visit</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr"/>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-16T23:15:06.498+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>visit</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr"/>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-16T23:15:06.535+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>visit</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr"/>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-16T23:15:32.308+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>